<commit_message>
Add shoulder-neck price gap threshold to watch pool
</commit_message>
<xml_diff>
--- a/backend/demo.xlsx
+++ b/backend/demo.xlsx
@@ -7,7 +7,7 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Demo" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="watch_pool" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -413,16 +413,17 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G3"/>
+  <dimension ref="A1:H3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="20" customWidth="1" min="1" max="1"/>
-    <col width="20" customWidth="1" min="2" max="2"/>
-    <col width="20" customWidth="1" min="3" max="3"/>
-    <col width="20" customWidth="1" min="4" max="4"/>
-    <col width="20" customWidth="1" min="5" max="5"/>
-    <col width="20" customWidth="1" min="6" max="6"/>
-    <col width="20" customWidth="1" min="7" max="7"/>
+    <col width="14" customWidth="1" min="1" max="1"/>
+    <col width="18" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="22" customWidth="1" min="5" max="5"/>
+    <col width="18" customWidth="1" min="6" max="6"/>
+    <col width="16" customWidth="1" min="7" max="7"/>
+    <col width="12" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -453,10 +454,15 @@
       </c>
       <c r="F1" t="inlineStr">
         <is>
+          <t>颈到肩最小价差</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
           <t>交易时间段</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>监控开关</t>
         </is>
@@ -484,12 +490,15 @@
       <c r="E2" t="n">
         <v>0</v>
       </c>
-      <c r="F2" t="inlineStr">
+      <c r="F2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G2" t="inlineStr">
         <is>
           <t>day,night</t>
         </is>
       </c>
-      <c r="G2" t="inlineStr">
+      <c r="H2" t="inlineStr">
         <is>
           <t>开启</t>
         </is>
@@ -517,12 +526,15 @@
       <c r="E3" t="n">
         <v>8</v>
       </c>
-      <c r="F3" t="inlineStr">
+      <c r="F3" t="n">
+        <v>4</v>
+      </c>
+      <c r="G3" t="inlineStr">
         <is>
           <t>day</t>
         </is>
       </c>
-      <c r="G3" t="inlineStr">
+      <c r="H3" t="inlineStr">
         <is>
           <t>开启</t>
         </is>

</xml_diff>